<commit_message>
data: publish 2026-10-07 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-07-182路.xlsx
+++ b/data/export/2026-10-07-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -632,32 +632,36 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -665,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -689,33 +693,37 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/11</t>
         </is>
       </c>
     </row>
@@ -743,32 +751,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,33 +812,37 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>3/11</t>
         </is>
       </c>
     </row>
@@ -854,32 +870,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:28</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,33 +931,37 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/11</t>
         </is>
       </c>
     </row>
@@ -998,7 +1022,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1037,7 +1061,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1048,7 +1072,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1133,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1159,7 +1183,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1244,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1294,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1355,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1405,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1466,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1516,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1577,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1603,7 +1627,685 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:44</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>1/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>3/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>1/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-07 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-07-182路.xlsx
+++ b/data/export/2026-10-07-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC64"/>
+  <dimension ref="A1:AC65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1308,17 +1308,17 @@
       </c>
       <c r="AA7" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="AB11" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC11" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="AB13" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC13" s="2" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2136,7 +2136,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2270,7 +2270,7 @@
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2617,17 +2617,17 @@
       </c>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="AB21" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC21" s="2" t="inlineStr">
@@ -3045,7 +3045,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="AB23" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC23" s="2" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3333,7 +3333,7 @@
       </c>
       <c r="AC24" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="Z25" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA25" s="2" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3918,17 +3918,17 @@
       </c>
       <c r="AA29" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -3993,7 +3993,7 @@
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC31" s="2" t="inlineStr">
@@ -4231,7 +4231,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -4270,7 +4270,7 @@
       </c>
       <c r="Z32" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA32" s="2" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="AC33" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P35" s="2" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="AA36" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB36" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC36" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="AB37" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC37" s="2" t="inlineStr">
@@ -4945,7 +4945,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC38" s="2" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5302,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -5659,7 +5659,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5708,7 +5708,7 @@
       </c>
       <c r="AB44" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC44" s="2" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P45" s="2" t="inlineStr">
@@ -5817,7 +5817,7 @@
       </c>
       <c r="Z45" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -6016,7 +6016,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6060,17 +6060,17 @@
       </c>
       <c r="AA47" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -6465,24 +6465,24 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>16:32</t>
+          <t>16:33</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>77分钟</t>
+          <t>78分钟</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -6492,7 +6492,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6541,7 +6541,7 @@
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
@@ -6611,7 +6611,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6650,7 +6650,7 @@
       </c>
       <c r="Z52" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="AA52" s="2" t="inlineStr">
@@ -6703,12 +6703,12 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>74分钟</t>
+          <t>75分钟</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="AB53" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC53" s="2" t="inlineStr">
@@ -6812,32 +6812,36 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>76分钟</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M54" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
           <t>06:11</t>
@@ -6845,7 +6849,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6869,17 +6873,17 @@
       </c>
       <c r="W54" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X54" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z54" s="2" t="inlineStr">
@@ -6889,17 +6893,17 @@
       </c>
       <c r="AA54" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>71.5</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
         <is>
-          <t>2/12</t>
+          <t>3/12</t>
         </is>
       </c>
     </row>
@@ -6960,7 +6964,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -7014,7 +7018,7 @@
       </c>
       <c r="AC55" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
         </is>
       </c>
     </row>
@@ -7075,7 +7079,7 @@
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P56" s="2" t="inlineStr">
@@ -7190,7 +7194,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
@@ -7305,7 +7309,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -7531,7 +7535,7 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -7646,7 +7650,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -7695,7 +7699,7 @@
       </c>
       <c r="AB61" s="2" t="inlineStr">
         <is>
-          <t>72.2</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC61" s="2" t="inlineStr">
@@ -7761,7 +7765,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -7810,7 +7814,7 @@
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
-          <t>70.6</t>
+          <t>70.8</t>
         </is>
       </c>
       <c r="AC62" s="2" t="inlineStr">
@@ -7876,7 +7880,7 @@
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P63" s="2" t="inlineStr">
@@ -7991,7 +7995,7 @@
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="P64" s="2" t="inlineStr">
@@ -8045,7 +8049,122 @@
       </c>
       <c r="AC64" s="2" t="inlineStr">
         <is>
-          <t>9/12</t>
+          <t>8/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr"/>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>16:32</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q65" s="2" t="inlineStr"/>
+      <c r="R65" s="2" t="inlineStr"/>
+      <c r="S65" s="2" t="inlineStr"/>
+      <c r="T65" s="2" t="inlineStr"/>
+      <c r="U65" s="2" t="inlineStr">
+        <is>
+          <t>17:25</t>
+        </is>
+      </c>
+      <c r="V65" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W65" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X65" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y65" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="AA65" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="AB65" s="2" t="inlineStr">
+        <is>
+          <t>70.5</t>
+        </is>
+      </c>
+      <c r="AC65" s="2" t="inlineStr">
+        <is>
+          <t>1/12</t>
         </is>
       </c>
     </row>

</xml_diff>